<commit_message>
feat: production pipeline validated and EBSERH 2020 acquired
</commit_message>
<xml_diff>
--- a/docs/imports/questions.xlsx
+++ b/docs/imports/questions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:W3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,6 +463,12 @@
       <c r="U1" t="str">
         <v>status</v>
       </c>
+      <c r="V1" t="str">
+        <v>package</v>
+      </c>
+      <c r="W1" t="str">
+        <v>package_version</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -528,6 +534,12 @@
       <c r="U2" t="str">
         <v>ACTIVE</v>
       </c>
+      <c r="V2" t="str">
+        <v>banco-de-questoes-enfermagem</v>
+      </c>
+      <c r="W2">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -578,10 +590,16 @@
       <c r="U3" t="str">
         <v>ACTIVE</v>
       </c>
+      <c r="V3" t="str">
+        <v>banco-de-questoes-enfermagem</v>
+      </c>
+      <c r="W3">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>